<commit_message>
feat: fulfillment kit for per-order .xlsm files; fix number formats in demo files
- docs/fulfillment/PANDUAN.md: workflow plus Prompt A (new order) and Prompt B
  (revision) for Claude, with fixed macro/spec conventions.
- scripts/fulfillment: generic build-xlsm.ps1 (spec.json + macro.bas -> .xlsm with
  Mulai/Hasil/Opsi/Petunjuk, named ranges, button), describe-xlsx.ps1, example and tests.
- Fix demo xlsx: number formats were read with the Indonesian locale
  (250000,0 instead of 250.000). Set via InvokeMember with en-US culture.
- Gitignore /pesanan/ (buyer data).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/demo/Contoh_Rekap_Penjualan.xlsx
+++ b/public/demo/Contoh_Rekap_Penjualan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Boy Manullang\Documents\1000 Code\bikinmacro\public\demo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{76EE88FF-F6D6-497D-A733-F62D81AA1A88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0CB48030-F4F0-43B0-B27F-DF863F18CD1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C7E78C27-8769-4DFD-B19D-9E8D21E47FBA}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{263A05FF-4C24-4D28-8AB1-23030338A4BE}"/>
   </bookViews>
   <sheets>
     <sheet name="Penjualan" sheetId="2" r:id="rId1"/>
@@ -114,8 +114,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="#.##0"/>
-    <numFmt numFmtId="165" formatCode="#,#00%"/>
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -170,9 +170,9 @@
   </cellStyleXfs>
   <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -489,7 +489,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{813DD4B0-4546-4A72-A469-C4E549099997}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{733911EE-070D-496E-ABE8-7C3FBF24F356}">
   <dimension ref="A1:H45"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -499,8 +499,8 @@
     <col min="4" max="4" width="8.44140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.21875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.5546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
@@ -1723,11 +1723,11 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BF6B46F-A08D-4A51-89E5-8666B55412BF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3C5DE85-EBC5-4921-86D9-4B5AE05D17A4}">
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.21875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.77734375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="62.77734375" customWidth="1"/>

</xml_diff>